<commit_message>
feat: PDF Roteiro Detalhado com altura dinâmica e fonte adaptativa por slots
- MinHeight em vez de Height nas linhas do diagrama: texto longo agora
  quebra para a linha seguinte em vez de ser clipado
- Font size calculado via Math.Clamp em função de slotsPerDay: trips com
  até 8 slots ficam com 7.5pt; acima disso reduz 0.3pt por slot extra (mín 6pt)
- Move scripts de importação para scripts/ e remove sys.path.insert desnecessário
- docs: IMPORT_GUIDE cobre formato .xls (xlrd), PROJECT_STRUCTURE documenta scripts/
- docs: remove TODO de PDF já resolvido

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Viagem Carretera Austral.xlsx
+++ b/Viagem Carretera Austral.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="451" documentId="13_ncr:1_{A7EC69DB-6D44-4749-9F82-125681D94D53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CEB83EF-55A5-424D-9BEA-0262C4905CB5}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B036FED7-6789-408A-AD16-AD775EE16E05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2310" yWindow="-120" windowWidth="36210" windowHeight="15720" tabRatio="769" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2310" yWindow="-120" windowWidth="36210" windowHeight="15720" tabRatio="769" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mapa" sheetId="55" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="343">
   <si>
     <t>dia</t>
   </si>
@@ -2066,12 +2066,6 @@
       </rPr>
       <t>10:00-12:00</t>
     </r>
-  </si>
-  <si>
-    <t>MOTORHOME</t>
-  </si>
-  <si>
-    <t>CARRO</t>
   </si>
   <si>
     <r>
@@ -3462,7 +3456,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="28">
+  <fills count="26">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3573,18 +3567,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -3626,7 +3608,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="29">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -3834,28 +3816,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </left>
-      <right style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </right>
-      <top style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -3870,118 +3830,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color theme="9" tint="-0.249977111117893"/>
-      </left>
-      <right style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </right>
-      <top style="medium">
-        <color theme="9" tint="-0.249977111117893"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </left>
-      <right style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </right>
-      <top style="medium">
-        <color theme="9" tint="-0.249977111117893"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </left>
-      <right style="medium">
-        <color theme="9" tint="-0.249977111117893"/>
-      </right>
-      <top style="medium">
-        <color theme="9" tint="-0.249977111117893"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="9" tint="-0.249977111117893"/>
-      </left>
-      <right style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </right>
-      <top style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </left>
-      <right style="medium">
-        <color theme="9" tint="-0.249977111117893"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="9" tint="-0.249977111117893"/>
-      </left>
-      <right style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </right>
-      <top style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </top>
-      <bottom style="medium">
-        <color theme="9" tint="-0.249977111117893"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </left>
-      <right style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </right>
-      <top style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </top>
-      <bottom style="medium">
-        <color theme="9" tint="-0.249977111117893"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </left>
-      <right style="medium">
-        <color theme="9" tint="-0.249977111117893"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color theme="9" tint="-0.249977111117893"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -3996,7 +3844,7 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="184">
+  <cellXfs count="146">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -4247,15 +4095,6 @@
     <xf numFmtId="0" fontId="27" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="10" fillId="9" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="9" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="10" fillId="9" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4265,261 +4104,150 @@
     <xf numFmtId="0" fontId="10" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="10" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="20" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="21" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="18" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="21" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="29" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="29" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="22" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="22" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="23" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="25" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="22" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="22" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="23" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="25" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="22" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="22" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="23" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="25" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="16" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="29" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="29" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="19" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="17" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="17" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="20" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="20" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="20" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4532,20 +4260,26 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="16" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="20" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -4881,270 +4615,270 @@
       <c r="J1" s="11"/>
     </row>
     <row r="2" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="104" t="s">
-        <v>275</v>
-      </c>
-      <c r="D2" s="100" t="s">
-        <v>248</v>
-      </c>
-      <c r="E2" s="102" t="s">
-        <v>249</v>
+      <c r="B2" s="96" t="s">
+        <v>273</v>
+      </c>
+      <c r="D2" s="92" t="s">
+        <v>246</v>
+      </c>
+      <c r="E2" s="94" t="s">
+        <v>247</v>
       </c>
       <c r="I2" s="11"/>
       <c r="J2" s="11"/>
     </row>
-    <row r="3" spans="2:10" s="97" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="96" t="s">
-        <v>230</v>
-      </c>
-      <c r="C3" s="96"/>
+    <row r="3" spans="2:10" s="89" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="88" t="s">
+        <v>228</v>
+      </c>
+      <c r="C3" s="88"/>
     </row>
     <row r="4" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="104" t="s">
-        <v>219</v>
-      </c>
-      <c r="D4" s="102" t="s">
-        <v>250</v>
+      <c r="B4" s="96" t="s">
+        <v>217</v>
+      </c>
+      <c r="D4" s="94" t="s">
+        <v>248</v>
       </c>
       <c r="G4" s="31"/>
       <c r="H4" s="31"/>
     </row>
-    <row r="5" spans="2:10" s="97" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="96" t="s">
+    <row r="5" spans="2:10" s="89" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="88" t="s">
+        <v>229</v>
+      </c>
+      <c r="C5" s="88"/>
+    </row>
+    <row r="6" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="96" t="s">
+        <v>218</v>
+      </c>
+      <c r="C6" s="88" t="s">
         <v>231</v>
       </c>
-      <c r="C5" s="96"/>
-    </row>
-    <row r="6" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="104" t="s">
-        <v>220</v>
-      </c>
-      <c r="C6" s="96" t="s">
-        <v>233</v>
-      </c>
-      <c r="D6" s="104" t="s">
-        <v>276</v>
-      </c>
-      <c r="E6" s="101" t="s">
+      <c r="D6" s="96" t="s">
+        <v>274</v>
+      </c>
+      <c r="E6" s="93" t="s">
         <v>94</v>
       </c>
       <c r="F6" s="31"/>
       <c r="G6" s="31"/>
       <c r="H6" s="31"/>
     </row>
-    <row r="7" spans="2:10" s="97" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="96" t="s">
-        <v>232</v>
-      </c>
-      <c r="C7" s="96"/>
+    <row r="7" spans="2:10" s="89" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="88" t="s">
+        <v>230</v>
+      </c>
+      <c r="C7" s="88"/>
     </row>
     <row r="8" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="104" t="s">
-        <v>277</v>
-      </c>
-      <c r="D8" s="102" t="s">
-        <v>251</v>
-      </c>
-      <c r="E8" s="97"/>
+      <c r="B8" s="96" t="s">
+        <v>275</v>
+      </c>
+      <c r="D8" s="94" t="s">
+        <v>249</v>
+      </c>
+      <c r="E8" s="89"/>
       <c r="G8" s="31"/>
       <c r="H8" s="31"/>
     </row>
-    <row r="9" spans="2:10" s="97" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="96" t="s">
+    <row r="9" spans="2:10" s="89" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="88" t="s">
+        <v>232</v>
+      </c>
+      <c r="C9" s="88"/>
+    </row>
+    <row r="10" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="96" t="s">
+        <v>276</v>
+      </c>
+      <c r="D10" s="92" t="s">
+        <v>55</v>
+      </c>
+      <c r="E10" s="94" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" s="89" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="88" t="s">
+        <v>233</v>
+      </c>
+      <c r="C11" s="88"/>
+    </row>
+    <row r="12" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="96" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" s="89" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="88" t="s">
         <v>234</v>
       </c>
-      <c r="C9" s="96"/>
-    </row>
-    <row r="10" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="104" t="s">
-        <v>278</v>
-      </c>
-      <c r="D10" s="100" t="s">
-        <v>55</v>
-      </c>
-      <c r="E10" s="102" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="11" spans="2:10" s="97" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="96" t="s">
+      <c r="C13" s="88"/>
+    </row>
+    <row r="14" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="96" t="s">
+        <v>220</v>
+      </c>
+      <c r="C14" s="88" t="s">
+        <v>244</v>
+      </c>
+      <c r="D14" s="96" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" s="89" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="88" t="s">
         <v>235</v>
       </c>
-      <c r="C11" s="96"/>
-    </row>
-    <row r="12" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="104" t="s">
+      <c r="D15" s="88" t="s">
+        <v>243</v>
+      </c>
+      <c r="I15" s="88"/>
+    </row>
+    <row r="16" spans="2:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="97" t="s">
+        <v>277</v>
+      </c>
+      <c r="C16" s="88" t="s">
+        <v>242</v>
+      </c>
+      <c r="D16" s="96" t="s">
+        <v>119</v>
+      </c>
+      <c r="J16" s="11"/>
+    </row>
+    <row r="17" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="88" t="s">
+        <v>236</v>
+      </c>
+      <c r="C17" s="89"/>
+      <c r="D17" s="89"/>
+      <c r="E17" s="89"/>
+      <c r="F17" s="89"/>
+      <c r="G17" s="89"/>
+      <c r="H17" s="89"/>
+      <c r="I17" s="89"/>
+      <c r="J17" s="11"/>
+    </row>
+    <row r="18" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="98" t="s">
+        <v>222</v>
+      </c>
+      <c r="C18" s="88" t="s">
+        <v>245</v>
+      </c>
+      <c r="D18" s="98" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="13" spans="2:10" s="97" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="96" t="s">
-        <v>236</v>
-      </c>
-      <c r="C13" s="96"/>
-    </row>
-    <row r="14" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="104" t="s">
-        <v>222</v>
-      </c>
-      <c r="C14" s="96" t="s">
-        <v>246</v>
-      </c>
-      <c r="D14" s="104" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="15" spans="2:10" s="97" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="96" t="s">
+      <c r="J18" s="11"/>
+    </row>
+    <row r="19" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="88" t="s">
         <v>237</v>
       </c>
-      <c r="D15" s="96" t="s">
-        <v>245</v>
-      </c>
-      <c r="I15" s="96"/>
-    </row>
-    <row r="16" spans="2:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="105" t="s">
-        <v>279</v>
-      </c>
-      <c r="C16" s="96" t="s">
-        <v>244</v>
-      </c>
-      <c r="D16" s="104" t="s">
-        <v>119</v>
-      </c>
-      <c r="J16" s="11"/>
-    </row>
-    <row r="17" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="96" t="s">
-        <v>238</v>
-      </c>
-      <c r="C17" s="97"/>
-      <c r="D17" s="97"/>
-      <c r="E17" s="97"/>
-      <c r="F17" s="97"/>
-      <c r="G17" s="97"/>
-      <c r="H17" s="97"/>
-      <c r="I17" s="97"/>
-      <c r="J17" s="11"/>
-    </row>
-    <row r="18" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="106" t="s">
-        <v>224</v>
-      </c>
-      <c r="C18" s="96" t="s">
-        <v>247</v>
-      </c>
-      <c r="D18" s="106" t="s">
-        <v>223</v>
-      </c>
-      <c r="J18" s="11"/>
-    </row>
-    <row r="19" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="96" t="s">
-        <v>239</v>
-      </c>
-      <c r="C19" s="97"/>
-      <c r="D19" s="97"/>
-      <c r="E19" s="97"/>
-      <c r="F19" s="97"/>
+      <c r="C19" s="89"/>
+      <c r="D19" s="89"/>
+      <c r="E19" s="89"/>
+      <c r="F19" s="89"/>
       <c r="I19" s="11"/>
       <c r="J19" s="11"/>
     </row>
     <row r="20" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="106" t="s">
-        <v>280</v>
-      </c>
-      <c r="D20" s="99" t="s">
+      <c r="B20" s="98" t="s">
+        <v>278</v>
+      </c>
+      <c r="D20" s="91" t="s">
         <v>58</v>
       </c>
-      <c r="E20" s="102" t="s">
-        <v>252</v>
+      <c r="E20" s="94" t="s">
+        <v>250</v>
       </c>
       <c r="I20" s="11"/>
       <c r="J20" s="11"/>
     </row>
     <row r="21" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="96" t="s">
+      <c r="B21" s="88" t="s">
+        <v>238</v>
+      </c>
+      <c r="C21" s="89"/>
+      <c r="D21" s="89"/>
+      <c r="E21" s="89"/>
+      <c r="F21" s="89"/>
+      <c r="G21" s="89"/>
+      <c r="H21" s="89"/>
+      <c r="I21" s="89"/>
+      <c r="J21" s="11"/>
+    </row>
+    <row r="22" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="98" t="s">
+        <v>279</v>
+      </c>
+      <c r="D22" s="91" t="s">
+        <v>251</v>
+      </c>
+      <c r="E22" s="94" t="s">
+        <v>252</v>
+      </c>
+      <c r="I22" s="11"/>
+    </row>
+    <row r="23" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="88" t="s">
+        <v>239</v>
+      </c>
+      <c r="E23" s="89"/>
+      <c r="F23" s="89"/>
+      <c r="G23" s="89"/>
+      <c r="H23" s="89"/>
+      <c r="I23" s="89"/>
+      <c r="J23" s="11"/>
+    </row>
+    <row r="24" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="98" t="s">
+        <v>223</v>
+      </c>
+      <c r="D24" s="94" t="s">
+        <v>253</v>
+      </c>
+      <c r="I24" s="11"/>
+    </row>
+    <row r="25" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="88" t="s">
         <v>240</v>
       </c>
-      <c r="C21" s="97"/>
-      <c r="D21" s="97"/>
-      <c r="E21" s="97"/>
-      <c r="F21" s="97"/>
-      <c r="G21" s="97"/>
-      <c r="H21" s="97"/>
-      <c r="I21" s="97"/>
-      <c r="J21" s="11"/>
-    </row>
-    <row r="22" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="106" t="s">
+      <c r="E25" s="89"/>
+      <c r="J25" s="11"/>
+    </row>
+    <row r="26" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="98" t="s">
+        <v>280</v>
+      </c>
+      <c r="D26" s="91" t="s">
+        <v>254</v>
+      </c>
+      <c r="E26" s="94" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="27" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="88" t="s">
+        <v>241</v>
+      </c>
+      <c r="C27" s="89"/>
+      <c r="D27" s="89"/>
+      <c r="E27" s="89"/>
+      <c r="F27" s="89"/>
+      <c r="G27" s="89"/>
+      <c r="H27" s="89"/>
+      <c r="I27" s="89"/>
+      <c r="J27" s="11"/>
+    </row>
+    <row r="28" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="98" t="s">
         <v>281</v>
       </c>
-      <c r="D22" s="99" t="s">
-        <v>253</v>
-      </c>
-      <c r="E22" s="102" t="s">
-        <v>254</v>
-      </c>
-      <c r="I22" s="11"/>
-    </row>
-    <row r="23" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="96" t="s">
-        <v>241</v>
-      </c>
-      <c r="E23" s="97"/>
-      <c r="F23" s="97"/>
-      <c r="G23" s="97"/>
-      <c r="H23" s="97"/>
-      <c r="I23" s="97"/>
-      <c r="J23" s="11"/>
-    </row>
-    <row r="24" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="106" t="s">
-        <v>225</v>
-      </c>
-      <c r="D24" s="102" t="s">
-        <v>255</v>
-      </c>
-      <c r="I24" s="11"/>
-    </row>
-    <row r="25" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="96" t="s">
-        <v>242</v>
-      </c>
-      <c r="E25" s="97"/>
-      <c r="J25" s="11"/>
-    </row>
-    <row r="26" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="106" t="s">
-        <v>282</v>
-      </c>
-      <c r="D26" s="99" t="s">
-        <v>256</v>
-      </c>
-      <c r="E26" s="102" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="27" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="96" t="s">
-        <v>243</v>
-      </c>
-      <c r="C27" s="97"/>
-      <c r="D27" s="97"/>
-      <c r="E27" s="97"/>
-      <c r="F27" s="97"/>
-      <c r="G27" s="97"/>
-      <c r="H27" s="97"/>
-      <c r="I27" s="97"/>
-      <c r="J27" s="11"/>
-    </row>
-    <row r="28" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="106" t="s">
-        <v>283</v>
-      </c>
-      <c r="D28" s="102" t="s">
+      <c r="D28" s="94" t="s">
         <v>62</v>
       </c>
       <c r="I28" s="11"/>
@@ -5207,11 +4941,11 @@
       <c r="L37" s="11"/>
     </row>
     <row r="38" spans="2:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I38" s="98"/>
+      <c r="I38" s="90"/>
     </row>
     <row r="39" spans="2:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H39" s="64"/>
-      <c r="I39" s="98"/>
+      <c r="I39" s="90"/>
       <c r="J39" s="11"/>
     </row>
   </sheetData>
@@ -5227,7 +4961,7 @@
     <tabColor rgb="FFFFC000"/>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
-  <dimension ref="B1:X22"/>
+  <dimension ref="B1:T23"/>
   <sheetFormatPr defaultRowHeight="35.1" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.28515625" style="11" customWidth="1"/>
@@ -5237,32 +4971,32 @@
     <col min="5" max="13" width="18.7109375" style="11" customWidth="1"/>
     <col min="14" max="14" width="13.140625" style="11" customWidth="1"/>
     <col min="15" max="15" width="20.7109375" style="31" customWidth="1"/>
-    <col min="16" max="17" width="4.85546875" style="11" customWidth="1"/>
-    <col min="18" max="26" width="18.7109375" style="11" customWidth="1"/>
-    <col min="27" max="16384" width="9.140625" style="11"/>
+    <col min="16" max="16" width="4.85546875" style="11" customWidth="1"/>
+    <col min="17" max="25" width="18.7109375" style="11" customWidth="1"/>
+    <col min="26" max="16384" width="9.140625" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:24" s="15" customFormat="1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:20" s="15" customFormat="1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="23" t="s">
         <v>16</v>
       </c>
       <c r="C1" s="24"/>
       <c r="D1" s="25"/>
-      <c r="E1" s="155" t="s">
+      <c r="E1" s="126" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="155"/>
-      <c r="G1" s="155"/>
-      <c r="H1" s="155"/>
-      <c r="I1" s="155"/>
-      <c r="J1" s="155"/>
-      <c r="K1" s="155"/>
-      <c r="L1" s="155"/>
-      <c r="M1" s="155"/>
-      <c r="N1" s="155"/>
-      <c r="O1" s="156"/>
-    </row>
-    <row r="2" spans="2:24" s="16" customFormat="1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F1" s="126"/>
+      <c r="G1" s="126"/>
+      <c r="H1" s="126"/>
+      <c r="I1" s="126"/>
+      <c r="J1" s="126"/>
+      <c r="K1" s="126"/>
+      <c r="L1" s="126"/>
+      <c r="M1" s="126"/>
+      <c r="N1" s="126"/>
+      <c r="O1" s="127"/>
+    </row>
+    <row r="2" spans="2:20" s="16" customFormat="1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="26" t="s">
         <v>1</v>
       </c>
@@ -5272,32 +5006,29 @@
       <c r="D2" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="157" t="s">
+      <c r="E2" s="128" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="157"/>
-      <c r="G2" s="157"/>
+      <c r="F2" s="128"/>
+      <c r="G2" s="128"/>
       <c r="H2" s="53" t="s">
         <v>35</v>
       </c>
-      <c r="I2" s="157" t="s">
+      <c r="I2" s="128" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="157"/>
-      <c r="K2" s="157"/>
-      <c r="L2" s="157"/>
-      <c r="M2" s="157"/>
+      <c r="J2" s="128"/>
+      <c r="K2" s="128"/>
+      <c r="L2" s="128"/>
+      <c r="M2" s="128"/>
       <c r="N2" s="27" t="s">
         <v>6</v>
       </c>
       <c r="O2" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="R2" s="26" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="3" spans="2:24" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="2:20" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="28">
         <v>45988</v>
       </c>
@@ -5308,11 +5039,15 @@
       <c r="D3" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="141" t="s">
-        <v>343</v>
-      </c>
-      <c r="J3" s="158"/>
-      <c r="K3" s="142"/>
+      <c r="E3" s="140"/>
+      <c r="F3" s="140"/>
+      <c r="G3" s="140"/>
+      <c r="H3" s="140"/>
+      <c r="I3" s="132" t="s">
+        <v>341</v>
+      </c>
+      <c r="J3" s="132"/>
+      <c r="K3" s="132"/>
       <c r="L3" s="82"/>
       <c r="M3" s="82"/>
       <c r="N3" s="82"/>
@@ -5320,7 +5055,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="4" spans="2:24" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:20" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="37">
         <f>B3+1</f>
         <v>45989</v>
@@ -5332,29 +5067,29 @@
       <c r="D4" s="52" t="s">
         <v>68</v>
       </c>
-      <c r="E4" s="147" t="s">
-        <v>226</v>
-      </c>
-      <c r="F4" s="148"/>
-      <c r="G4" s="149"/>
+      <c r="E4" s="129" t="s">
+        <v>224</v>
+      </c>
+      <c r="F4" s="129"/>
+      <c r="G4" s="129"/>
       <c r="H4" s="55" t="s">
         <v>36</v>
       </c>
-      <c r="I4" s="140" t="s">
-        <v>294</v>
-      </c>
-      <c r="J4" s="140"/>
-      <c r="K4" s="140"/>
-      <c r="L4" s="141" t="s">
-        <v>295</v>
-      </c>
-      <c r="M4" s="142"/>
+      <c r="I4" s="132" t="s">
+        <v>292</v>
+      </c>
+      <c r="J4" s="132"/>
+      <c r="K4" s="132"/>
+      <c r="L4" s="132" t="s">
+        <v>293</v>
+      </c>
+      <c r="M4" s="132"/>
       <c r="N4" s="82"/>
       <c r="O4" s="58" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="2:24" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:20" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="37">
         <f t="shared" ref="B5:B18" si="1">B4+1</f>
         <v>45990</v>
@@ -5367,7 +5102,7 @@
         <v>69</v>
       </c>
       <c r="E5" s="80" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="F5" s="81" t="s">
         <v>148</v>
@@ -5378,32 +5113,29 @@
       <c r="H5" s="83" t="s">
         <v>36</v>
       </c>
-      <c r="I5" s="151" t="s">
+      <c r="I5" s="131" t="s">
         <v>150</v>
       </c>
-      <c r="J5" s="152"/>
-      <c r="K5" s="147" t="s">
+      <c r="J5" s="131"/>
+      <c r="K5" s="129" t="s">
         <v>59</v>
       </c>
-      <c r="L5" s="148"/>
-      <c r="M5" s="149"/>
+      <c r="L5" s="129"/>
+      <c r="M5" s="129"/>
       <c r="N5" s="82"/>
       <c r="O5" s="59" t="s">
         <v>59</v>
       </c>
-      <c r="P5" s="143" t="s">
-        <v>218</v>
+      <c r="Q5" s="107" t="s">
+        <v>166</v>
       </c>
       <c r="R5" s="129" t="s">
-        <v>166</v>
-      </c>
-      <c r="S5" s="139" t="s">
         <v>156</v>
       </c>
-      <c r="T5" s="139"/>
-      <c r="U5" s="139"/>
-    </row>
-    <row r="6" spans="2:24" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S5" s="129"/>
+      <c r="T5" s="129"/>
+    </row>
+    <row r="6" spans="2:20" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="37">
         <f>B5+1</f>
         <v>45991</v>
@@ -5415,18 +5147,18 @@
       <c r="D6" s="52" t="s">
         <v>70</v>
       </c>
-      <c r="E6" s="159" t="s">
+      <c r="E6" s="129" t="s">
         <v>151</v>
       </c>
-      <c r="F6" s="159"/>
-      <c r="G6" s="159"/>
+      <c r="F6" s="129"/>
+      <c r="G6" s="129"/>
       <c r="H6" s="83" t="s">
         <v>36</v>
       </c>
-      <c r="I6" s="160" t="s">
-        <v>227</v>
-      </c>
-      <c r="J6" s="161"/>
+      <c r="I6" s="141" t="s">
+        <v>225</v>
+      </c>
+      <c r="J6" s="141"/>
       <c r="K6" s="81" t="s">
         <v>152</v>
       </c>
@@ -5440,9 +5172,8 @@
       <c r="O6" s="59" t="s">
         <v>61</v>
       </c>
-      <c r="P6" s="143"/>
-    </row>
-    <row r="7" spans="2:24" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="2:20" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="37">
         <f t="shared" si="1"/>
         <v>45992</v>
@@ -5454,45 +5185,27 @@
       <c r="D7" s="52" t="s">
         <v>71</v>
       </c>
-      <c r="E7" s="162" t="s">
+      <c r="E7" s="131" t="s">
         <v>127</v>
       </c>
-      <c r="F7" s="162"/>
-      <c r="G7" s="139" t="s">
+      <c r="F7" s="131"/>
+      <c r="G7" s="129" t="s">
         <v>142</v>
       </c>
-      <c r="H7" s="139"/>
-      <c r="I7" s="139"/>
-      <c r="J7" s="139"/>
-      <c r="K7" s="139"/>
-      <c r="L7" s="162" t="s">
+      <c r="H7" s="129"/>
+      <c r="I7" s="129"/>
+      <c r="J7" s="129"/>
+      <c r="K7" s="129"/>
+      <c r="L7" s="131" t="s">
         <v>128</v>
       </c>
-      <c r="M7" s="162"/>
+      <c r="M7" s="131"/>
       <c r="N7" s="82"/>
       <c r="O7" s="59" t="s">
         <v>61</v>
       </c>
-      <c r="P7" s="143"/>
-      <c r="R7" s="121" t="s">
-        <v>167</v>
-      </c>
-      <c r="S7" s="81" t="s">
-        <v>290</v>
-      </c>
-      <c r="T7" s="139" t="s">
-        <v>289</v>
-      </c>
-      <c r="U7" s="139"/>
-      <c r="V7" s="139"/>
-      <c r="W7" s="81" t="s">
-        <v>291</v>
-      </c>
-      <c r="X7" s="81" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="8" spans="2:24" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="2:20" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="37">
         <f t="shared" si="1"/>
         <v>45993</v>
@@ -5504,19 +5217,19 @@
       <c r="D8" s="52" t="s">
         <v>72</v>
       </c>
-      <c r="E8" s="147" t="s">
-        <v>229</v>
-      </c>
-      <c r="F8" s="148"/>
-      <c r="G8" s="149"/>
-      <c r="H8" s="92" t="s">
+      <c r="E8" s="129" t="s">
+        <v>227</v>
+      </c>
+      <c r="F8" s="129"/>
+      <c r="G8" s="129"/>
+      <c r="H8" s="83" t="s">
         <v>36</v>
       </c>
-      <c r="I8" s="163" t="s">
-        <v>228</v>
-      </c>
-      <c r="J8" s="164"/>
-      <c r="K8" s="164"/>
+      <c r="I8" s="134" t="s">
+        <v>226</v>
+      </c>
+      <c r="J8" s="134"/>
+      <c r="K8" s="134"/>
       <c r="L8" s="81" t="s">
         <v>154</v>
       </c>
@@ -5527,451 +5240,440 @@
       <c r="O8" s="59" t="s">
         <v>59</v>
       </c>
-      <c r="P8" s="143"/>
-    </row>
-    <row r="9" spans="2:24" ht="35.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="84">
+    </row>
+    <row r="9" spans="2:20" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="37">
         <f t="shared" si="1"/>
         <v>45994</v>
       </c>
-      <c r="C9" s="85">
+      <c r="C9" s="36">
         <f t="shared" si="0"/>
         <v>45994</v>
       </c>
-      <c r="D9" s="86" t="s">
+      <c r="D9" s="52" t="s">
         <v>73</v>
       </c>
-      <c r="E9" s="139" t="s">
+      <c r="E9" s="129" t="s">
         <v>156</v>
       </c>
-      <c r="F9" s="139"/>
-      <c r="G9" s="139"/>
-      <c r="H9" s="92" t="s">
+      <c r="F9" s="129"/>
+      <c r="G9" s="129"/>
+      <c r="H9" s="83" t="s">
         <v>36</v>
       </c>
       <c r="I9" s="82" t="s">
         <v>59</v>
       </c>
-      <c r="J9" s="146" t="s">
+      <c r="J9" s="131" t="s">
         <v>157</v>
       </c>
-      <c r="K9" s="146"/>
-      <c r="L9" s="93" t="s">
+      <c r="K9" s="131"/>
+      <c r="L9" s="81" t="s">
         <v>158</v>
       </c>
-      <c r="M9" s="93" t="s">
+      <c r="M9" s="81" t="s">
         <v>159</v>
       </c>
-      <c r="N9" s="91"/>
+      <c r="N9" s="82"/>
       <c r="O9" s="59" t="s">
         <v>60</v>
       </c>
-      <c r="P9" s="143"/>
-      <c r="R9" s="121" t="s">
-        <v>101</v>
-      </c>
-      <c r="S9" s="144" t="s">
-        <v>183</v>
-      </c>
-      <c r="T9" s="144"/>
-      <c r="U9" s="145"/>
-      <c r="V9" s="81" t="s">
-        <v>292</v>
-      </c>
-      <c r="W9" s="82" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="10" spans="2:24" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="110">
+    </row>
+    <row r="10" spans="2:20" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="142">
         <f t="shared" si="1"/>
         <v>45995</v>
       </c>
-      <c r="C10" s="111">
+      <c r="C10" s="102">
         <f t="shared" si="0"/>
         <v>45995</v>
       </c>
-      <c r="D10" s="112" t="s">
+      <c r="D10" s="103" t="s">
         <v>74</v>
       </c>
-      <c r="E10" s="113" t="s">
-        <v>324</v>
-      </c>
-      <c r="F10" s="174" t="s">
+      <c r="E10" s="143" t="s">
+        <v>322</v>
+      </c>
+      <c r="F10" s="144" t="s">
         <v>216</v>
       </c>
-      <c r="G10" s="174"/>
-      <c r="H10" s="114" t="s">
+      <c r="G10" s="144"/>
+      <c r="H10" s="106" t="s">
         <v>36</v>
       </c>
-      <c r="I10" s="113" t="s">
+      <c r="I10" s="143" t="s">
         <v>214</v>
       </c>
-      <c r="J10" s="115" t="s">
+      <c r="J10" s="104" t="s">
         <v>60</v>
       </c>
-      <c r="K10" s="116" t="s">
+      <c r="K10" s="105" t="s">
         <v>148</v>
       </c>
-      <c r="L10" s="116" t="s">
+      <c r="L10" s="105" t="s">
         <v>149</v>
       </c>
-      <c r="M10" s="115" t="s">
+      <c r="M10" s="104" t="s">
         <v>101</v>
       </c>
-      <c r="N10" s="115"/>
-      <c r="O10" s="94" t="s">
+      <c r="N10" s="104"/>
+      <c r="O10" s="87" t="s">
         <v>101</v>
       </c>
-      <c r="P10" s="171" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="11" spans="2:24" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="117">
+    </row>
+    <row r="11" spans="2:20" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="142">
         <f t="shared" si="1"/>
         <v>45996</v>
       </c>
-      <c r="C11" s="118">
+      <c r="C11" s="102">
         <f t="shared" si="0"/>
         <v>45996</v>
       </c>
-      <c r="D11" s="119" t="s">
+      <c r="D11" s="103" t="s">
         <v>75</v>
       </c>
-      <c r="E11" s="168" t="s">
+      <c r="E11" s="125" t="s">
         <v>145</v>
       </c>
-      <c r="F11" s="168"/>
-      <c r="G11" s="168"/>
-      <c r="H11" s="168"/>
-      <c r="I11" s="168"/>
-      <c r="J11" s="168"/>
-      <c r="K11" s="121" t="s">
+      <c r="F11" s="125"/>
+      <c r="G11" s="125"/>
+      <c r="H11" s="125"/>
+      <c r="I11" s="125"/>
+      <c r="J11" s="125"/>
+      <c r="K11" s="105" t="s">
         <v>158</v>
       </c>
-      <c r="L11" s="121" t="s">
+      <c r="L11" s="105" t="s">
         <v>159</v>
       </c>
-      <c r="M11" s="120" t="s">
+      <c r="M11" s="104" t="s">
         <v>60</v>
       </c>
-      <c r="N11" s="120"/>
-      <c r="O11" s="90" t="s">
+      <c r="N11" s="104"/>
+      <c r="O11" s="87" t="s">
         <v>60</v>
       </c>
-      <c r="P11" s="172"/>
-    </row>
-    <row r="12" spans="2:24" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="117">
+    </row>
+    <row r="12" spans="2:20" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="142">
         <f t="shared" si="1"/>
         <v>45997</v>
       </c>
-      <c r="C12" s="118">
+      <c r="C12" s="102">
         <f t="shared" si="0"/>
         <v>45997</v>
       </c>
-      <c r="D12" s="119" t="s">
+      <c r="D12" s="103" t="s">
         <v>76</v>
       </c>
-      <c r="E12" s="121" t="s">
+      <c r="E12" s="105" t="s">
         <v>129</v>
       </c>
-      <c r="F12" s="121" t="s">
+      <c r="F12" s="105" t="s">
         <v>130</v>
       </c>
-      <c r="G12" s="121" t="s">
+      <c r="G12" s="105" t="s">
         <v>131</v>
       </c>
-      <c r="H12" s="122" t="s">
+      <c r="H12" s="106" t="s">
         <v>36</v>
       </c>
-      <c r="I12" s="168" t="s">
-        <v>288</v>
-      </c>
-      <c r="J12" s="168"/>
-      <c r="K12" s="168"/>
-      <c r="L12" s="168" t="s">
+      <c r="I12" s="125" t="s">
+        <v>286</v>
+      </c>
+      <c r="J12" s="125"/>
+      <c r="K12" s="125"/>
+      <c r="L12" s="125" t="s">
         <v>51</v>
       </c>
-      <c r="M12" s="168"/>
-      <c r="N12" s="120"/>
-      <c r="O12" s="90" t="s">
+      <c r="M12" s="125"/>
+      <c r="N12" s="104"/>
+      <c r="O12" s="87" t="s">
         <v>51</v>
       </c>
-      <c r="P12" s="172"/>
-    </row>
-    <row r="13" spans="2:24" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="117">
+    </row>
+    <row r="13" spans="2:20" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="142">
         <f>B12+1</f>
         <v>45998</v>
       </c>
-      <c r="C13" s="118">
+      <c r="C13" s="102">
         <f t="shared" si="0"/>
         <v>45998</v>
       </c>
-      <c r="D13" s="119" t="s">
+      <c r="D13" s="103" t="s">
         <v>77</v>
       </c>
-      <c r="E13" s="121" t="s">
+      <c r="E13" s="105" t="s">
         <v>132</v>
       </c>
-      <c r="F13" s="121" t="s">
+      <c r="F13" s="105" t="s">
         <v>133</v>
       </c>
-      <c r="G13" s="121" t="s">
+      <c r="G13" s="105" t="s">
         <v>134</v>
       </c>
-      <c r="H13" s="122" t="s">
+      <c r="H13" s="106" t="s">
         <v>36</v>
       </c>
-      <c r="I13" s="168" t="s">
+      <c r="I13" s="125" t="s">
         <v>209</v>
       </c>
-      <c r="J13" s="168"/>
-      <c r="K13" s="168"/>
-      <c r="L13" s="168"/>
-      <c r="M13" s="168"/>
-      <c r="N13" s="120"/>
-      <c r="O13" s="90" t="s">
+      <c r="J13" s="125"/>
+      <c r="K13" s="125"/>
+      <c r="L13" s="125"/>
+      <c r="M13" s="125"/>
+      <c r="N13" s="104"/>
+      <c r="O13" s="87" t="s">
         <v>94</v>
       </c>
-      <c r="P13" s="172"/>
-    </row>
-    <row r="14" spans="2:24" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="117">
+    </row>
+    <row r="14" spans="2:20" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="142">
         <f t="shared" si="1"/>
         <v>45999</v>
       </c>
-      <c r="C14" s="118">
+      <c r="C14" s="102">
         <f t="shared" si="0"/>
         <v>45999</v>
       </c>
-      <c r="D14" s="119" t="s">
+      <c r="D14" s="103" t="s">
         <v>78</v>
       </c>
-      <c r="E14" s="121" t="s">
+      <c r="E14" s="105" t="s">
         <v>135</v>
       </c>
-      <c r="F14" s="121" t="s">
+      <c r="F14" s="105" t="s">
         <v>136</v>
       </c>
-      <c r="G14" s="121" t="s">
+      <c r="G14" s="105" t="s">
         <v>137</v>
       </c>
-      <c r="H14" s="122" t="s">
+      <c r="H14" s="106" t="s">
         <v>36</v>
       </c>
-      <c r="I14" s="168" t="s">
+      <c r="I14" s="125" t="s">
         <v>144</v>
       </c>
-      <c r="J14" s="168"/>
-      <c r="K14" s="168"/>
-      <c r="L14" s="168" t="s">
+      <c r="J14" s="125"/>
+      <c r="K14" s="125"/>
+      <c r="L14" s="125" t="s">
         <v>48</v>
       </c>
-      <c r="M14" s="168"/>
-      <c r="N14" s="120"/>
-      <c r="O14" s="90" t="s">
+      <c r="M14" s="125"/>
+      <c r="N14" s="104"/>
+      <c r="O14" s="87" t="s">
         <v>48</v>
       </c>
-      <c r="P14" s="172"/>
-    </row>
-    <row r="15" spans="2:24" s="57" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="117">
+    </row>
+    <row r="15" spans="2:20" s="57" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="142">
         <f t="shared" si="1"/>
         <v>46000</v>
       </c>
-      <c r="C15" s="118">
+      <c r="C15" s="102">
         <f t="shared" si="0"/>
         <v>46000</v>
       </c>
-      <c r="D15" s="119" t="s">
+      <c r="D15" s="103" t="s">
         <v>79</v>
       </c>
-      <c r="E15" s="121" t="s">
+      <c r="E15" s="105" t="s">
         <v>138</v>
       </c>
-      <c r="F15" s="168" t="s">
+      <c r="F15" s="125" t="s">
         <v>179</v>
       </c>
-      <c r="G15" s="168"/>
-      <c r="H15" s="122" t="s">
+      <c r="G15" s="125"/>
+      <c r="H15" s="106" t="s">
         <v>36</v>
       </c>
-      <c r="I15" s="121" t="s">
+      <c r="I15" s="105" t="s">
         <v>139</v>
       </c>
-      <c r="J15" s="121" t="s">
+      <c r="J15" s="105" t="s">
         <v>140</v>
       </c>
-      <c r="K15" s="168" t="s">
+      <c r="K15" s="125" t="s">
         <v>160</v>
       </c>
-      <c r="L15" s="168"/>
-      <c r="M15" s="168"/>
-      <c r="N15" s="120"/>
-      <c r="O15" s="90" t="s">
+      <c r="L15" s="125"/>
+      <c r="M15" s="125"/>
+      <c r="N15" s="104"/>
+      <c r="O15" s="87" t="s">
         <v>52</v>
       </c>
-      <c r="P15" s="172"/>
-      <c r="Q15" s="11"/>
-      <c r="R15" s="121" t="s">
-        <v>163</v>
-      </c>
-      <c r="S15" s="165" t="s">
-        <v>182</v>
-      </c>
-      <c r="T15" s="166"/>
-      <c r="U15" s="166"/>
-      <c r="V15" s="167"/>
-    </row>
-    <row r="16" spans="2:24" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="117">
+      <c r="P15" s="11"/>
+    </row>
+    <row r="16" spans="2:20" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="142">
         <f>B15+1</f>
         <v>46001</v>
       </c>
-      <c r="C16" s="118">
+      <c r="C16" s="102">
         <f t="shared" si="0"/>
         <v>46001</v>
       </c>
-      <c r="D16" s="119" t="s">
+      <c r="D16" s="103" t="s">
         <v>87</v>
       </c>
-      <c r="E16" s="121" t="s">
+      <c r="E16" s="105" t="s">
         <v>141</v>
       </c>
-      <c r="F16" s="153" t="s">
+      <c r="F16" s="125" t="s">
         <v>143</v>
       </c>
-      <c r="G16" s="154"/>
-      <c r="H16" s="122" t="s">
+      <c r="G16" s="125"/>
+      <c r="H16" s="106" t="s">
         <v>36</v>
       </c>
-      <c r="I16" s="123" t="s">
+      <c r="I16" s="105" t="s">
         <v>146</v>
       </c>
-      <c r="J16" s="123" t="s">
+      <c r="J16" s="105" t="s">
         <v>147</v>
       </c>
-      <c r="K16" s="123" t="s">
-        <v>285</v>
-      </c>
-      <c r="L16" s="123" t="s">
+      <c r="K16" s="105" t="s">
+        <v>283</v>
+      </c>
+      <c r="L16" s="105" t="s">
+        <v>282</v>
+      </c>
+      <c r="M16" s="105" t="s">
         <v>284</v>
       </c>
-      <c r="M16" s="123" t="s">
-        <v>286</v>
-      </c>
-      <c r="N16" s="120"/>
-      <c r="O16" s="90" t="s">
+      <c r="N16" s="104"/>
+      <c r="O16" s="87" t="s">
         <v>60</v>
       </c>
-      <c r="P16" s="172"/>
-    </row>
-    <row r="17" spans="2:18" s="31" customFormat="1" ht="35.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="124">
+    </row>
+    <row r="17" spans="2:17" s="31" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="142">
         <f t="shared" si="1"/>
         <v>46002</v>
       </c>
-      <c r="C17" s="125">
+      <c r="C17" s="102">
         <f t="shared" si="0"/>
         <v>46002</v>
       </c>
-      <c r="D17" s="126" t="s">
+      <c r="D17" s="103" t="s">
         <v>88</v>
       </c>
-      <c r="E17" s="127"/>
-      <c r="F17" s="169" t="s">
+      <c r="E17" s="104"/>
+      <c r="F17" s="144" t="s">
         <v>215</v>
       </c>
-      <c r="G17" s="169"/>
-      <c r="H17" s="128" t="s">
+      <c r="G17" s="144"/>
+      <c r="H17" s="106" t="s">
         <v>36</v>
       </c>
-      <c r="I17" s="170" t="s">
+      <c r="I17" s="145" t="s">
         <v>202</v>
       </c>
-      <c r="J17" s="170"/>
-      <c r="K17" s="170" t="s">
+      <c r="J17" s="145"/>
+      <c r="K17" s="145" t="s">
         <v>201</v>
       </c>
-      <c r="L17" s="170"/>
-      <c r="M17" s="170"/>
-      <c r="N17" s="127"/>
-      <c r="O17" s="95" t="s">
+      <c r="L17" s="145"/>
+      <c r="M17" s="145"/>
+      <c r="N17" s="104"/>
+      <c r="O17" s="58" t="s">
         <v>67</v>
       </c>
-      <c r="P17" s="173"/>
+      <c r="P17" s="11"/>
       <c r="Q17" s="11"/>
-      <c r="R17" s="11"/>
-    </row>
-    <row r="18" spans="2:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="87">
+    </row>
+    <row r="18" spans="2:17" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="84">
         <f t="shared" si="1"/>
         <v>46003</v>
       </c>
-      <c r="C18" s="88">
+      <c r="C18" s="85">
         <f t="shared" si="0"/>
         <v>46003</v>
       </c>
-      <c r="D18" s="89" t="s">
+      <c r="D18" s="86" t="s">
         <v>89</v>
       </c>
-      <c r="E18" s="120"/>
-      <c r="F18" s="120"/>
-      <c r="G18" s="150" t="s">
-        <v>344</v>
-      </c>
-      <c r="H18" s="150"/>
-      <c r="I18" s="150"/>
-    </row>
-    <row r="19" spans="2:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E18" s="139"/>
+      <c r="F18" s="139"/>
+      <c r="G18" s="130" t="s">
+        <v>342</v>
+      </c>
+      <c r="H18" s="130"/>
+      <c r="I18" s="130"/>
+    </row>
+    <row r="19" spans="2:17" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="11"/>
       <c r="C19" s="11"/>
       <c r="D19" s="11"/>
       <c r="O19" s="11"/>
     </row>
-    <row r="20" spans="2:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="11"/>
+    <row r="20" spans="2:17" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="26" t="s">
+        <v>285</v>
+      </c>
       <c r="C20" s="11"/>
       <c r="D20" s="11"/>
       <c r="O20" s="11"/>
     </row>
-    <row r="21" spans="2:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
+    <row r="21" spans="2:17" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="105" t="s">
+        <v>167</v>
+      </c>
+      <c r="C21" s="81" t="s">
+        <v>288</v>
+      </c>
+      <c r="D21" s="129" t="s">
+        <v>287</v>
+      </c>
+      <c r="E21" s="129"/>
+      <c r="F21" s="129"/>
+      <c r="G21" s="81" t="s">
+        <v>289</v>
+      </c>
+      <c r="H21" s="81" t="s">
+        <v>153</v>
+      </c>
       <c r="O21" s="11"/>
     </row>
-    <row r="22" spans="2:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="O22" s="11"/>
+    <row r="22" spans="2:17" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="105" t="s">
+        <v>101</v>
+      </c>
+      <c r="C22" s="133" t="s">
+        <v>183</v>
+      </c>
+      <c r="D22" s="133"/>
+      <c r="E22" s="134"/>
+      <c r="F22" s="81" t="s">
+        <v>290</v>
+      </c>
+      <c r="G22" s="82" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="23" spans="2:17" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="105" t="s">
+        <v>163</v>
+      </c>
+      <c r="C23" s="122" t="s">
+        <v>182</v>
+      </c>
+      <c r="D23" s="123"/>
+      <c r="E23" s="123"/>
+      <c r="F23" s="124"/>
+      <c r="G23" s="57"/>
+      <c r="H23" s="57"/>
     </row>
   </sheetData>
-  <mergeCells count="38">
-    <mergeCell ref="S15:V15"/>
-    <mergeCell ref="L14:M14"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="K15:M15"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="K17:M17"/>
-    <mergeCell ref="P10:P17"/>
-    <mergeCell ref="E11:J11"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="I13:M13"/>
-    <mergeCell ref="I14:K14"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="E1:O1"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="I2:M2"/>
-    <mergeCell ref="I3:K3"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="I6:J6"/>
+  <mergeCells count="36">
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="I4:K4"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="R5:T5"/>
+    <mergeCell ref="C22:E22"/>
     <mergeCell ref="E9:G9"/>
     <mergeCell ref="J9:K9"/>
     <mergeCell ref="E4:G4"/>
@@ -5984,12 +5686,25 @@
     <mergeCell ref="L7:M7"/>
     <mergeCell ref="E8:G8"/>
     <mergeCell ref="I8:K8"/>
-    <mergeCell ref="T7:V7"/>
-    <mergeCell ref="I4:K4"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="S5:U5"/>
-    <mergeCell ref="P5:P9"/>
-    <mergeCell ref="S9:U9"/>
+    <mergeCell ref="E1:O1"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="I2:M2"/>
+    <mergeCell ref="I3:K3"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="L14:M14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="K15:M15"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="K17:M17"/>
+    <mergeCell ref="E11:J11"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="I13:M13"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="F10:G10"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" scale="58" orientation="portrait" r:id="rId1"/>
@@ -6098,10 +5813,10 @@
       <c r="F6" s="74"/>
     </row>
     <row r="7" spans="1:6" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="175" t="s">
+      <c r="A7" s="135" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="176"/>
+      <c r="B7" s="136"/>
       <c r="C7" s="63" t="s">
         <v>169</v>
       </c>
@@ -6124,10 +5839,10 @@
       <c r="F8" s="74"/>
     </row>
     <row r="9" spans="1:6" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="175" t="s">
+      <c r="A9" s="135" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="176"/>
+      <c r="B9" s="136"/>
       <c r="C9" s="63" t="s">
         <v>171</v>
       </c>
@@ -6164,10 +5879,10 @@
       <c r="F11" s="74"/>
     </row>
     <row r="12" spans="1:6" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="175" t="s">
+      <c r="A12" s="135" t="s">
         <v>94</v>
       </c>
-      <c r="B12" s="176"/>
+      <c r="B12" s="136"/>
       <c r="C12" s="63" t="s">
         <v>178</v>
       </c>
@@ -6204,10 +5919,10 @@
       <c r="F14" s="74"/>
     </row>
     <row r="15" spans="1:6" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="175" t="s">
+      <c r="A15" s="135" t="s">
         <v>48</v>
       </c>
-      <c r="B15" s="176"/>
+      <c r="B15" s="136"/>
       <c r="C15" s="63" t="s">
         <v>184</v>
       </c>
@@ -6216,20 +5931,20 @@
       <c r="F15" s="74"/>
     </row>
     <row r="16" spans="1:6" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="175" t="s">
+      <c r="A16" s="135" t="s">
         <v>164</v>
       </c>
-      <c r="B16" s="176"/>
+      <c r="B16" s="136"/>
       <c r="C16" s="63"/>
       <c r="D16" s="74"/>
       <c r="E16" s="74"/>
       <c r="F16" s="74"/>
     </row>
     <row r="17" spans="1:6" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="175" t="s">
+      <c r="A17" s="135" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="176"/>
+      <c r="B17" s="136"/>
       <c r="C17" s="63"/>
       <c r="D17" s="74"/>
       <c r="E17" s="74"/>
@@ -6260,10 +5975,10 @@
       <c r="F19" s="74"/>
     </row>
     <row r="20" spans="1:6" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="177" t="s">
+      <c r="A20" s="137" t="s">
         <v>101</v>
       </c>
-      <c r="B20" s="178"/>
+      <c r="B20" s="138"/>
       <c r="C20" s="63" t="s">
         <v>168</v>
       </c>
@@ -6284,10 +5999,10 @@
       <c r="F21" s="74"/>
     </row>
     <row r="22" spans="1:6" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="177" t="s">
+      <c r="A22" s="137" t="s">
         <v>166</v>
       </c>
-      <c r="B22" s="178"/>
+      <c r="B22" s="138"/>
       <c r="C22" s="63"/>
       <c r="D22" s="74"/>
       <c r="E22" s="74"/>
@@ -6318,10 +6033,10 @@
       <c r="F24" s="74"/>
     </row>
     <row r="25" spans="1:6" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="177" t="s">
+      <c r="A25" s="137" t="s">
         <v>61</v>
       </c>
-      <c r="B25" s="178"/>
+      <c r="B25" s="138"/>
       <c r="C25" s="63"/>
       <c r="D25" s="74"/>
       <c r="E25" s="74"/>
@@ -6340,30 +6055,30 @@
       <c r="F26" s="74"/>
     </row>
     <row r="27" spans="1:6" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="177" t="s">
+      <c r="A27" s="137" t="s">
         <v>62</v>
       </c>
-      <c r="B27" s="178"/>
+      <c r="B27" s="138"/>
       <c r="C27" s="63"/>
       <c r="D27" s="74"/>
       <c r="E27" s="74"/>
       <c r="F27" s="74"/>
     </row>
     <row r="28" spans="1:6" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="175" t="s">
+      <c r="A28" s="135" t="s">
         <v>164</v>
       </c>
-      <c r="B28" s="176"/>
+      <c r="B28" s="136"/>
       <c r="C28" s="63"/>
       <c r="D28" s="74"/>
       <c r="E28" s="74"/>
       <c r="F28" s="74"/>
     </row>
     <row r="29" spans="1:6" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="175" t="s">
+      <c r="A29" s="135" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="176"/>
+      <c r="B29" s="136"/>
       <c r="C29" s="63"/>
       <c r="D29" s="74"/>
       <c r="E29" s="74"/>
@@ -6379,18 +6094,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A16:B16"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A16:B16"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6432,7 +6147,7 @@
     </row>
     <row r="2" spans="1:5" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="B2" s="60" t="s">
         <v>60</v>
@@ -6442,22 +6157,22 @@
       </c>
       <c r="D2" s="60"/>
       <c r="E2" s="29" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="22" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B3" s="60" t="s">
         <v>60</v>
       </c>
       <c r="C3" s="60" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D3" s="60"/>
       <c r="E3" s="29" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -6694,18 +6409,18 @@
     </row>
     <row r="3" spans="1:2" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="22" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B3" s="29" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="22" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B4" s="29" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -6849,7 +6564,7 @@
         <v>206</v>
       </c>
       <c r="B22" s="29" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="23" spans="1:2" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -7009,11 +6724,11 @@
       <c r="E1" s="33" t="s">
         <v>197</v>
       </c>
-      <c r="F1" s="179" t="s">
+      <c r="F1" s="118" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="179"/>
-      <c r="H1" s="179"/>
+      <c r="G1" s="118"/>
+      <c r="H1" s="118"/>
       <c r="I1" s="43" t="s">
         <v>13</v>
       </c>
@@ -7047,7 +6762,7 @@
       <c r="B2" s="51" t="s">
         <v>93</v>
       </c>
-      <c r="C2" s="180" t="s">
+      <c r="C2" s="119" t="s">
         <v>26</v>
       </c>
       <c r="D2" s="54" t="s">
@@ -7091,28 +6806,28 @@
       </c>
       <c r="Q2" s="42"/>
     </row>
-    <row r="3" spans="1:17" s="109" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" s="101" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="38" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="51" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="180"/>
+      <c r="C3" s="119"/>
       <c r="D3" s="54" t="s">
         <v>33</v>
       </c>
       <c r="E3" s="41" t="s">
         <v>189</v>
       </c>
-      <c r="F3" s="107" t="s">
+      <c r="F3" s="99" t="s">
         <v>200</v>
       </c>
-      <c r="G3" s="107" t="s">
-        <v>297</v>
-      </c>
-      <c r="H3" s="107" t="s">
-        <v>296</v>
+      <c r="G3" s="99" t="s">
+        <v>295</v>
+      </c>
+      <c r="H3" s="99" t="s">
+        <v>294</v>
       </c>
       <c r="I3" s="39">
         <v>152.38999999999999</v>
@@ -7139,29 +6854,29 @@
         <f>O3</f>
         <v>304.77999999999997</v>
       </c>
-      <c r="Q3" s="108"/>
-    </row>
-    <row r="4" spans="1:17" s="109" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q3" s="100"/>
+    </row>
+    <row r="4" spans="1:17" s="101" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="38" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="51" t="s">
         <v>91</v>
       </c>
-      <c r="C4" s="180"/>
-      <c r="D4" s="130" t="s">
-        <v>298</v>
-      </c>
-      <c r="E4" s="103" t="s">
-        <v>299</v>
-      </c>
-      <c r="F4" s="107" t="s">
+      <c r="C4" s="119"/>
+      <c r="D4" s="108" t="s">
+        <v>296</v>
+      </c>
+      <c r="E4" s="95" t="s">
+        <v>297</v>
+      </c>
+      <c r="F4" s="99" t="s">
         <v>189</v>
       </c>
-      <c r="G4" s="107" t="s">
+      <c r="G4" s="99" t="s">
         <v>189</v>
       </c>
-      <c r="H4" s="107" t="s">
+      <c r="H4" s="99" t="s">
         <v>189</v>
       </c>
       <c r="I4" s="48">
@@ -7187,16 +6902,16 @@
         <v>234.09667439999998</v>
       </c>
       <c r="P4" s="39" t="s">
-        <v>326</v>
-      </c>
-      <c r="Q4" s="108"/>
+        <v>324</v>
+      </c>
+      <c r="Q4" s="100"/>
     </row>
     <row r="5" spans="1:17" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="38"/>
       <c r="B5" s="51" t="s">
         <v>91</v>
       </c>
-      <c r="C5" s="180"/>
+      <c r="C5" s="119"/>
       <c r="D5" s="78" t="s">
         <v>203</v>
       </c>
@@ -7240,23 +6955,23 @@
     <row r="6" spans="1:17" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="38"/>
       <c r="B6" s="51" t="s">
+        <v>261</v>
+      </c>
+      <c r="C6" s="119"/>
+      <c r="D6" s="78" t="s">
         <v>263</v>
       </c>
-      <c r="C6" s="180"/>
-      <c r="D6" s="78" t="s">
+      <c r="E6" s="95" t="s">
+        <v>262</v>
+      </c>
+      <c r="F6" s="56" t="s">
+        <v>264</v>
+      </c>
+      <c r="G6" s="56" t="s">
         <v>265</v>
       </c>
-      <c r="E6" s="103" t="s">
-        <v>264</v>
-      </c>
-      <c r="F6" s="56" t="s">
+      <c r="H6" s="56" t="s">
         <v>266</v>
-      </c>
-      <c r="G6" s="56" t="s">
-        <v>267</v>
-      </c>
-      <c r="H6" s="56" t="s">
-        <v>268</v>
       </c>
       <c r="I6" s="44">
         <v>675</v>
@@ -7283,68 +6998,68 @@
       <c r="P6" s="39"/>
       <c r="Q6" s="42"/>
     </row>
-    <row r="7" spans="1:17" s="137" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="131" t="s">
+    <row r="7" spans="1:17" s="115" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="109" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="51" t="s">
-        <v>262</v>
-      </c>
-      <c r="C7" s="180"/>
-      <c r="D7" s="130" t="s">
+        <v>260</v>
+      </c>
+      <c r="C7" s="119"/>
+      <c r="D7" s="108" t="s">
+        <v>268</v>
+      </c>
+      <c r="E7" s="110" t="s">
+        <v>267</v>
+      </c>
+      <c r="F7" s="111" t="s">
+        <v>269</v>
+      </c>
+      <c r="G7" s="111" t="s">
         <v>270</v>
       </c>
-      <c r="E7" s="132" t="s">
-        <v>269</v>
-      </c>
-      <c r="F7" s="133" t="s">
-        <v>271</v>
-      </c>
-      <c r="G7" s="133" t="s">
-        <v>272</v>
-      </c>
-      <c r="H7" s="133" t="s">
-        <v>322</v>
-      </c>
-      <c r="I7" s="134">
+      <c r="H7" s="111" t="s">
+        <v>320</v>
+      </c>
+      <c r="I7" s="112">
         <v>327127</v>
       </c>
-      <c r="J7" s="134"/>
+      <c r="J7" s="112"/>
       <c r="K7" s="40">
         <v>1</v>
       </c>
       <c r="L7" s="41">
         <v>1</v>
       </c>
-      <c r="M7" s="134">
+      <c r="M7" s="112">
         <v>352127</v>
       </c>
-      <c r="N7" s="135">
+      <c r="N7" s="113">
         <f>CLP*(1+IOF_Wise)</f>
         <v>6.5026853999999995E-3</v>
       </c>
-      <c r="O7" s="135">
+      <c r="O7" s="113">
         <f t="shared" ref="O7" si="6">M7*N7</f>
         <v>2289.7711018457999</v>
       </c>
-      <c r="P7" s="135">
+      <c r="P7" s="113">
         <f>O7</f>
         <v>2289.7711018457999</v>
       </c>
-      <c r="Q7" s="136"/>
-    </row>
-    <row r="8" spans="1:17" s="109" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q7" s="114"/>
+    </row>
+    <row r="8" spans="1:17" s="101" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="38" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="51" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="180"/>
+      <c r="C8" s="119"/>
       <c r="D8" s="54" t="s">
         <v>85</v>
       </c>
-      <c r="E8" s="103" t="s">
+      <c r="E8" s="95" t="s">
         <v>192</v>
       </c>
       <c r="F8" s="54" t="s">
@@ -7353,7 +7068,7 @@
       <c r="G8" s="54" t="s">
         <v>198</v>
       </c>
-      <c r="H8" s="107" t="s">
+      <c r="H8" s="99" t="s">
         <v>189</v>
       </c>
       <c r="I8" s="44">
@@ -7382,8 +7097,8 @@
         <f>837.05*N8</f>
         <v>4941.8979992999994</v>
       </c>
-      <c r="Q8" s="108" t="s">
-        <v>318</v>
+      <c r="Q8" s="100" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="9" spans="1:17" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -7393,7 +7108,7 @@
       <c r="B9" s="51" t="s">
         <v>90</v>
       </c>
-      <c r="C9" s="180"/>
+      <c r="C9" s="119"/>
       <c r="D9" s="78" t="s">
         <v>189</v>
       </c>
@@ -7439,23 +7154,23 @@
       <c r="B10" s="51" t="s">
         <v>186</v>
       </c>
-      <c r="C10" s="181" t="s">
+      <c r="C10" s="120" t="s">
         <v>28</v>
       </c>
       <c r="D10" s="56" t="s">
         <v>188</v>
       </c>
       <c r="E10" s="77" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="F10" s="56" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="G10" s="56" t="s">
-        <v>303</v>
-      </c>
-      <c r="H10" s="107" t="s">
-        <v>308</v>
+        <v>301</v>
+      </c>
+      <c r="H10" s="99" t="s">
+        <v>306</v>
       </c>
       <c r="I10" s="44">
         <v>44</v>
@@ -7486,28 +7201,28 @@
       </c>
       <c r="Q10" s="42"/>
     </row>
-    <row r="11" spans="1:17" s="109" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" s="101" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="38" t="s">
         <v>7</v>
       </c>
       <c r="B11" s="51" t="s">
+        <v>298</v>
+      </c>
+      <c r="C11" s="121"/>
+      <c r="D11" s="99" t="s">
+        <v>299</v>
+      </c>
+      <c r="E11" s="95" t="s">
+        <v>321</v>
+      </c>
+      <c r="F11" s="99" t="s">
+        <v>308</v>
+      </c>
+      <c r="G11" s="99" t="s">
         <v>300</v>
       </c>
-      <c r="C11" s="182"/>
-      <c r="D11" s="107" t="s">
-        <v>301</v>
-      </c>
-      <c r="E11" s="103" t="s">
-        <v>323</v>
-      </c>
-      <c r="F11" s="107" t="s">
-        <v>310</v>
-      </c>
-      <c r="G11" s="107" t="s">
+      <c r="H11" s="99" t="s">
         <v>302</v>
-      </c>
-      <c r="H11" s="107" t="s">
-        <v>304</v>
       </c>
       <c r="I11" s="44">
         <v>85</v>
@@ -7534,30 +7249,30 @@
       <c r="P11" s="39" t="s">
         <v>213</v>
       </c>
-      <c r="Q11" s="108"/>
-    </row>
-    <row r="12" spans="1:17" s="109" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q11" s="100"/>
+    </row>
+    <row r="12" spans="1:17" s="101" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="38" t="s">
         <v>7</v>
       </c>
       <c r="B12" s="51" t="s">
-        <v>327</v>
-      </c>
-      <c r="C12" s="182"/>
-      <c r="D12" s="107" t="s">
-        <v>316</v>
-      </c>
-      <c r="E12" s="103" t="s">
-        <v>320</v>
-      </c>
-      <c r="F12" s="107" t="s">
-        <v>311</v>
-      </c>
-      <c r="G12" s="107" t="s">
-        <v>317</v>
-      </c>
-      <c r="H12" s="107" t="s">
-        <v>308</v>
+        <v>325</v>
+      </c>
+      <c r="C12" s="121"/>
+      <c r="D12" s="99" t="s">
+        <v>314</v>
+      </c>
+      <c r="E12" s="95" t="s">
+        <v>318</v>
+      </c>
+      <c r="F12" s="99" t="s">
+        <v>309</v>
+      </c>
+      <c r="G12" s="99" t="s">
+        <v>315</v>
+      </c>
+      <c r="H12" s="99" t="s">
+        <v>306</v>
       </c>
       <c r="I12" s="44">
         <v>77</v>
@@ -7586,30 +7301,30 @@
       <c r="P12" s="39" t="s">
         <v>213</v>
       </c>
-      <c r="Q12" s="108"/>
-    </row>
-    <row r="13" spans="1:17" s="109" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q12" s="100"/>
+    </row>
+    <row r="13" spans="1:17" s="101" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="38" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="51" t="s">
-        <v>273</v>
-      </c>
-      <c r="C13" s="182"/>
-      <c r="D13" s="107" t="s">
+        <v>271</v>
+      </c>
+      <c r="C13" s="121"/>
+      <c r="D13" s="99" t="s">
+        <v>304</v>
+      </c>
+      <c r="E13" s="95" t="s">
+        <v>319</v>
+      </c>
+      <c r="F13" s="99" t="s">
+        <v>310</v>
+      </c>
+      <c r="G13" s="99" t="s">
+        <v>305</v>
+      </c>
+      <c r="H13" s="99" t="s">
         <v>306</v>
-      </c>
-      <c r="E13" s="103" t="s">
-        <v>321</v>
-      </c>
-      <c r="F13" s="107" t="s">
-        <v>312</v>
-      </c>
-      <c r="G13" s="107" t="s">
-        <v>307</v>
-      </c>
-      <c r="H13" s="107" t="s">
-        <v>308</v>
       </c>
       <c r="I13" s="44">
         <v>150</v>
@@ -7638,30 +7353,30 @@
       <c r="P13" s="39" t="s">
         <v>213</v>
       </c>
-      <c r="Q13" s="108"/>
-    </row>
-    <row r="14" spans="1:17" s="109" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q13" s="100"/>
+    </row>
+    <row r="14" spans="1:17" s="101" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="38" t="s">
         <v>7</v>
       </c>
       <c r="B14" s="51" t="s">
+        <v>326</v>
+      </c>
+      <c r="C14" s="121"/>
+      <c r="D14" s="99" t="s">
+        <v>327</v>
+      </c>
+      <c r="E14" s="95" t="s">
+        <v>329</v>
+      </c>
+      <c r="F14" s="99" t="s">
+        <v>311</v>
+      </c>
+      <c r="G14" s="99" t="s">
         <v>328</v>
       </c>
-      <c r="C14" s="182"/>
-      <c r="D14" s="107" t="s">
-        <v>329</v>
-      </c>
-      <c r="E14" s="103" t="s">
-        <v>331</v>
-      </c>
-      <c r="F14" s="107" t="s">
-        <v>313</v>
-      </c>
-      <c r="G14" s="107" t="s">
-        <v>330</v>
-      </c>
-      <c r="H14" s="107" t="s">
-        <v>308</v>
+      <c r="H14" s="99" t="s">
+        <v>306</v>
       </c>
       <c r="I14" s="39">
         <v>499.18</v>
@@ -7688,30 +7403,30 @@
         <f>O14</f>
         <v>499.18</v>
       </c>
-      <c r="Q14" s="108"/>
-    </row>
-    <row r="15" spans="1:17" s="109" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q14" s="100"/>
+    </row>
+    <row r="15" spans="1:17" s="101" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="38" t="s">
         <v>7</v>
       </c>
       <c r="B15" s="51" t="s">
-        <v>305</v>
-      </c>
-      <c r="C15" s="182"/>
-      <c r="D15" s="107" t="s">
-        <v>301</v>
-      </c>
-      <c r="E15" s="103" t="s">
-        <v>323</v>
-      </c>
-      <c r="F15" s="107" t="s">
-        <v>314</v>
-      </c>
-      <c r="G15" s="107" t="s">
+        <v>303</v>
+      </c>
+      <c r="C15" s="121"/>
+      <c r="D15" s="99" t="s">
+        <v>299</v>
+      </c>
+      <c r="E15" s="95" t="s">
+        <v>321</v>
+      </c>
+      <c r="F15" s="99" t="s">
+        <v>312</v>
+      </c>
+      <c r="G15" s="99" t="s">
+        <v>300</v>
+      </c>
+      <c r="H15" s="99" t="s">
         <v>302</v>
-      </c>
-      <c r="H15" s="107" t="s">
-        <v>304</v>
       </c>
       <c r="I15" s="44">
         <v>85</v>
@@ -7738,7 +7453,7 @@
       <c r="P15" s="39" t="s">
         <v>213</v>
       </c>
-      <c r="Q15" s="108"/>
+      <c r="Q15" s="100"/>
     </row>
     <row r="16" spans="1:17" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="38" t="s">
@@ -7747,21 +7462,21 @@
       <c r="B16" s="51" t="s">
         <v>187</v>
       </c>
-      <c r="C16" s="182"/>
+      <c r="C16" s="121"/>
       <c r="D16" s="56" t="s">
         <v>188</v>
       </c>
       <c r="E16" s="77" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="F16" s="56" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="G16" s="56" t="s">
-        <v>303</v>
-      </c>
-      <c r="H16" s="107" t="s">
-        <v>308</v>
+        <v>301</v>
+      </c>
+      <c r="H16" s="99" t="s">
+        <v>306</v>
       </c>
       <c r="I16" s="44">
         <v>44</v>
@@ -7792,23 +7507,23 @@
       </c>
       <c r="Q16" s="42"/>
     </row>
-    <row r="17" spans="1:17" s="109" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:17" s="101" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="38" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="51" t="s">
-        <v>335</v>
-      </c>
-      <c r="C17" s="182"/>
-      <c r="D17" s="130"/>
+        <v>333</v>
+      </c>
+      <c r="C17" s="121"/>
+      <c r="D17" s="108"/>
       <c r="E17" s="77"/>
-      <c r="F17" s="107" t="s">
+      <c r="F17" s="99" t="s">
         <v>189</v>
       </c>
-      <c r="G17" s="107" t="s">
+      <c r="G17" s="99" t="s">
         <v>189</v>
       </c>
-      <c r="H17" s="107" t="s">
+      <c r="H17" s="99" t="s">
         <v>189</v>
       </c>
       <c r="I17" s="48">
@@ -7834,29 +7549,29 @@
         <v>117.04833719999999</v>
       </c>
       <c r="P17" s="39"/>
-      <c r="Q17" s="108"/>
-    </row>
-    <row r="18" spans="1:17" s="109" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q17" s="100"/>
+    </row>
+    <row r="18" spans="1:17" s="101" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="38" t="s">
         <v>7</v>
       </c>
       <c r="B18" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="C18" s="138"/>
-      <c r="D18" s="130" t="s">
+        <v>331</v>
+      </c>
+      <c r="C18" s="116"/>
+      <c r="D18" s="108" t="s">
+        <v>330</v>
+      </c>
+      <c r="E18" s="77" t="s">
         <v>332</v>
       </c>
-      <c r="E18" s="77" t="s">
-        <v>334</v>
-      </c>
-      <c r="F18" s="107" t="s">
+      <c r="F18" s="99" t="s">
         <v>189</v>
       </c>
-      <c r="G18" s="107" t="s">
+      <c r="G18" s="99" t="s">
         <v>189</v>
       </c>
-      <c r="H18" s="107" t="s">
+      <c r="H18" s="99" t="s">
         <v>189</v>
       </c>
       <c r="I18" s="48">
@@ -7882,21 +7597,21 @@
         <v>117.04833719999999</v>
       </c>
       <c r="P18" s="39"/>
-      <c r="Q18" s="108"/>
-    </row>
-    <row r="19" spans="1:17" s="109" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q18" s="100"/>
+    </row>
+    <row r="19" spans="1:17" s="101" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="38" t="s">
         <v>7</v>
       </c>
       <c r="B19" s="51" t="s">
-        <v>336</v>
-      </c>
-      <c r="C19" s="138"/>
-      <c r="D19" s="130"/>
+        <v>334</v>
+      </c>
+      <c r="C19" s="116"/>
+      <c r="D19" s="108"/>
       <c r="E19" s="41"/>
-      <c r="F19" s="107"/>
-      <c r="G19" s="107"/>
-      <c r="H19" s="107"/>
+      <c r="F19" s="99"/>
+      <c r="G19" s="99"/>
+      <c r="H19" s="99"/>
       <c r="I19" s="48"/>
       <c r="J19" s="48"/>
       <c r="K19" s="40"/>
@@ -7905,21 +7620,21 @@
       <c r="N19" s="39"/>
       <c r="O19" s="39"/>
       <c r="P19" s="39"/>
-      <c r="Q19" s="108"/>
-    </row>
-    <row r="20" spans="1:17" s="109" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q19" s="100"/>
+    </row>
+    <row r="20" spans="1:17" s="101" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="38" t="s">
         <v>7</v>
       </c>
       <c r="B20" s="51" t="s">
-        <v>337</v>
-      </c>
-      <c r="C20" s="138"/>
-      <c r="D20" s="130"/>
+        <v>335</v>
+      </c>
+      <c r="C20" s="116"/>
+      <c r="D20" s="108"/>
       <c r="E20" s="41"/>
-      <c r="F20" s="107"/>
-      <c r="G20" s="107"/>
-      <c r="H20" s="107"/>
+      <c r="F20" s="99"/>
+      <c r="G20" s="99"/>
+      <c r="H20" s="99"/>
       <c r="I20" s="48"/>
       <c r="J20" s="48"/>
       <c r="K20" s="40"/>
@@ -7928,21 +7643,21 @@
       <c r="N20" s="39"/>
       <c r="O20" s="39"/>
       <c r="P20" s="39"/>
-      <c r="Q20" s="108"/>
-    </row>
-    <row r="21" spans="1:17" s="109" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q20" s="100"/>
+    </row>
+    <row r="21" spans="1:17" s="101" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="38" t="s">
         <v>7</v>
       </c>
       <c r="B21" s="51" t="s">
-        <v>338</v>
-      </c>
-      <c r="C21" s="138"/>
-      <c r="D21" s="130"/>
+        <v>336</v>
+      </c>
+      <c r="C21" s="116"/>
+      <c r="D21" s="108"/>
       <c r="E21" s="41"/>
-      <c r="F21" s="107"/>
-      <c r="G21" s="107"/>
-      <c r="H21" s="107"/>
+      <c r="F21" s="99"/>
+      <c r="G21" s="99"/>
+      <c r="H21" s="99"/>
       <c r="I21" s="48"/>
       <c r="J21" s="48"/>
       <c r="K21" s="40"/>
@@ -7951,21 +7666,21 @@
       <c r="N21" s="39"/>
       <c r="O21" s="39"/>
       <c r="P21" s="39"/>
-      <c r="Q21" s="108"/>
-    </row>
-    <row r="22" spans="1:17" s="109" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q21" s="100"/>
+    </row>
+    <row r="22" spans="1:17" s="101" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="38" t="s">
         <v>7</v>
       </c>
       <c r="B22" s="51" t="s">
-        <v>339</v>
-      </c>
-      <c r="C22" s="138"/>
-      <c r="D22" s="130"/>
+        <v>337</v>
+      </c>
+      <c r="C22" s="116"/>
+      <c r="D22" s="108"/>
       <c r="E22" s="41"/>
-      <c r="F22" s="107"/>
-      <c r="G22" s="107"/>
-      <c r="H22" s="107"/>
+      <c r="F22" s="99"/>
+      <c r="G22" s="99"/>
+      <c r="H22" s="99"/>
       <c r="I22" s="48"/>
       <c r="J22" s="48"/>
       <c r="K22" s="40"/>
@@ -7974,29 +7689,29 @@
       <c r="N22" s="39"/>
       <c r="O22" s="39"/>
       <c r="P22" s="39"/>
-      <c r="Q22" s="108"/>
+      <c r="Q22" s="100"/>
     </row>
     <row r="23" spans="1:17" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="38" t="s">
         <v>7</v>
       </c>
       <c r="B23" s="51" t="s">
-        <v>333</v>
-      </c>
-      <c r="C23" s="138"/>
-      <c r="D23" s="130" t="s">
+        <v>331</v>
+      </c>
+      <c r="C23" s="116"/>
+      <c r="D23" s="108" t="s">
+        <v>330</v>
+      </c>
+      <c r="E23" s="77" t="s">
         <v>332</v>
       </c>
-      <c r="E23" s="77" t="s">
-        <v>334</v>
-      </c>
-      <c r="F23" s="107" t="s">
+      <c r="F23" s="99" t="s">
         <v>189</v>
       </c>
-      <c r="G23" s="107" t="s">
+      <c r="G23" s="99" t="s">
         <v>189</v>
       </c>
-      <c r="H23" s="107" t="s">
+      <c r="H23" s="99" t="s">
         <v>189</v>
       </c>
       <c r="I23" s="48">
@@ -8027,7 +7742,7 @@
     <row r="24" spans="1:17" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="38"/>
       <c r="B24" s="51"/>
-      <c r="C24" s="180" t="s">
+      <c r="C24" s="119" t="s">
         <v>34</v>
       </c>
       <c r="D24" s="78" t="s">
@@ -8058,7 +7773,7 @@
     <row r="25" spans="1:17" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="38"/>
       <c r="B25" s="51"/>
-      <c r="C25" s="180"/>
+      <c r="C25" s="119"/>
       <c r="D25" s="78" t="s">
         <v>189</v>
       </c>
@@ -8087,7 +7802,7 @@
     <row r="26" spans="1:17" s="9" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="38"/>
       <c r="B26" s="51"/>
-      <c r="C26" s="180"/>
+      <c r="C26" s="119"/>
       <c r="D26" s="78" t="s">
         <v>189</v>
       </c>
@@ -8120,7 +7835,7 @@
       <c r="B27" s="51" t="s">
         <v>190</v>
       </c>
-      <c r="C27" s="180" t="s">
+      <c r="C27" s="119" t="s">
         <v>29</v>
       </c>
       <c r="D27" s="78" t="s">
@@ -8169,7 +7884,7 @@
       <c r="B28" s="51" t="s">
         <v>31</v>
       </c>
-      <c r="C28" s="180"/>
+      <c r="C28" s="119"/>
       <c r="D28" s="78" t="s">
         <v>189</v>
       </c>
@@ -8216,7 +7931,7 @@
       <c r="B29" s="51" t="s">
         <v>32</v>
       </c>
-      <c r="C29" s="180"/>
+      <c r="C29" s="119"/>
       <c r="D29" s="78" t="s">
         <v>189</v>
       </c>
@@ -8305,19 +8020,19 @@
       <c r="F33" s="1"/>
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
-      <c r="M33" s="183" t="s">
+      <c r="M33" s="117" t="s">
         <v>24</v>
       </c>
-      <c r="N33" s="183"/>
+      <c r="N33" s="117"/>
       <c r="O33" s="45">
         <v>5.66</v>
       </c>
     </row>
     <row r="34" spans="2:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M34" s="183" t="s">
+      <c r="M34" s="117" t="s">
         <v>30</v>
       </c>
-      <c r="N34" s="183"/>
+      <c r="N34" s="117"/>
       <c r="O34" s="46">
         <v>6.234E-3</v>
       </c>
@@ -8332,19 +8047,19 @@
       </c>
     </row>
     <row r="36" spans="2:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M36" s="183" t="s">
+      <c r="M36" s="117" t="s">
         <v>25</v>
       </c>
-      <c r="N36" s="183"/>
+      <c r="N36" s="117"/>
       <c r="O36" s="47">
         <v>6.3799999999999996E-2</v>
       </c>
     </row>
     <row r="37" spans="2:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M37" s="183" t="s">
+      <c r="M37" s="117" t="s">
         <v>185</v>
       </c>
-      <c r="N37" s="183"/>
+      <c r="N37" s="117"/>
       <c r="O37" s="47">
         <f>(3.5+0.81)/100</f>
         <v>4.3100000000000006E-2</v>
@@ -8352,15 +8067,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="C2:C9"/>
+    <mergeCell ref="C10:C17"/>
+    <mergeCell ref="C24:C26"/>
+    <mergeCell ref="C27:C29"/>
     <mergeCell ref="M37:N37"/>
     <mergeCell ref="M33:N33"/>
     <mergeCell ref="M34:N34"/>
     <mergeCell ref="M36:N36"/>
     <mergeCell ref="F1:H1"/>
-    <mergeCell ref="C2:C9"/>
-    <mergeCell ref="C10:C17"/>
-    <mergeCell ref="C24:C26"/>
-    <mergeCell ref="C27:C29"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E10" r:id="rId1" xr:uid="{00000000-0004-0000-0A00-000001000000}"/>

</xml_diff>